<commit_message>
feat(saff-study): publish specification and test suite v2.2
</commit_message>
<xml_diff>
--- a/output/xlsx/DelecaoExtracoes--GT-.xlsx
+++ b/output/xlsx/DelecaoExtracoes--GT-.xlsx
@@ -71,7 +71,7 @@
     <t xml:space="preserve">Precondition: </t>
   </si>
   <si>
-    <t>Usuario deve estar logado no servidor ; 705 extracoes ja foram realizadas (pasta “EXTRACT_FILE_IPP320_AKIRA”)</t>
+    <t>Usuario deve estar logado no servidor e extrator como administrador ; 705 extracoes ja foram realizadas (pasta “EXTRACT_FILE_IPP320_AKIRA”)</t>
   </si>
   <si>
     <t>#</t>
@@ -263,7 +263,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="91.4296875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="116.5390625" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="79.53515625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
feat(saff-study): publish specification and test suite v2.4
</commit_message>
<xml_diff>
--- a/output/xlsx/DelecaoExtracoes--GT-.xlsx
+++ b/output/xlsx/DelecaoExtracoes--GT-.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="51">
   <si>
     <t xml:space="preserve">System: </t>
   </si>
@@ -71,7 +71,7 @@
     <t xml:space="preserve">Precondition: </t>
   </si>
   <si>
-    <t>Usuario deve estar logado no servidor e extrator como administrador ; 705 extracoes ja foram realizadas (pasta “EXTRACT_FILE_IPP320_AKIRA”)</t>
+    <t>Usuário deve estar logado no servidor e extrator como administrador ; 705 extrações já realizadas (pasta “EXTRACT_FILE_IPP320_AKIRA”)</t>
   </si>
   <si>
     <t>#</t>
@@ -92,25 +92,25 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>administrador: seleciona o check box referente a extracao referente ao numero serial 12311PP30154516”</t>
+    <t>administrador: seleciona o check box referente a extração referente ao número serial 12311PP30154516”</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>SYSTEM marca selecao com um tick</t>
-  </si>
-  <si>
-    <t>administrador: pressiona o botao “Delete extractions”</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe uma mensagem pop-up solicitando a confirmação da delecao</t>
-  </si>
-  <si>
-    <t>administrador: confirma delecao</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe a lista de extracoes com 704 entradas</t>
+    <t>SYSTEM marca seleção com um tick</t>
+  </si>
+  <si>
+    <t>administrador: pressiona o botão “Delete extractions”</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe uma mensagem pop-up solicitando a confirmação da deleção</t>
+  </si>
+  <si>
+    <t>administrador: confirma deleção</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe a lista de extrações com 704 entradas</t>
   </si>
   <si>
     <t xml:space="preserve">Postcondition: </t>
@@ -119,10 +119,10 @@
     <t>TC2</t>
   </si>
   <si>
-    <t>Alternative Flow 1: Cancela delecao</t>
-  </si>
-  <si>
-    <t>administrador: cancela delecao</t>
+    <t>Alternative Flow 1: Cancela deleção</t>
+  </si>
+  <si>
+    <t>administrador: cancela deleção</t>
   </si>
   <si>
     <t>SYSTEM fecha janela pop-up</t>
@@ -131,43 +131,40 @@
     <t>TC3</t>
   </si>
   <si>
-    <t>Alternative Flow 2: Realiza Filtro e delecao</t>
+    <t>Alternative Flow 2: Realiza Filtro e deleção</t>
   </si>
   <si>
     <t>administrador: seleciona combo box referente ao filtro por “State”</t>
   </si>
   <si>
-    <t>SYSTEM exibe opcoes “Activated”, “Alert Interruption”, “Deactivated”, “Mockup” e “Error”</t>
-  </si>
-  <si>
-    <t>administrador: seleciona opcao “Activated” no campo de filtro “State”</t>
-  </si>
-  <si>
-    <t>SYSTEM atualiza pagina mostrando 608 extracoes</t>
-  </si>
-  <si>
-    <t>administrador: seleciona o check box que marca todas extracoes para delecao</t>
-  </si>
-  <si>
-    <t>SYSTEM marca todas extracoes após o filtro com um tick</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe uma mensagem pop-up solicitando a confirmacao da delecao</t>
-  </si>
-  <si>
-    <t>SYSTEM exibe a lista de extracoes com 96 entradas</t>
+    <t>SYSTEM exibe opções “Activated”, “Alert Interruption”, “Deactivated”, “Mockup” e “Error”</t>
+  </si>
+  <si>
+    <t>administrador: seleciona opção “Activated” no campo de filtro “State”</t>
+  </si>
+  <si>
+    <t>SYSTEM atualiza página mostrando 608 extrações</t>
+  </si>
+  <si>
+    <t>administrador: seleciona o check box que marca todas extrações para deleção</t>
+  </si>
+  <si>
+    <t>SYSTEM marca todas extrações após o filtro com um tick</t>
+  </si>
+  <si>
+    <t>SYSTEM exibe a lista de extrações com 96 entradas</t>
   </si>
   <si>
     <t>TC4</t>
   </si>
   <si>
-    <t>Alternative Flow 3: Deleta todas extracoes</t>
+    <t>Alternative Flow 3: Deleta todas extrações</t>
   </si>
   <si>
     <t>SYSTEM marca o check box com um tick</t>
   </si>
   <si>
-    <t>SYSTEM exibe uma mensagem pop-up indicando que nao existem extracoes para serem deletadas</t>
+    <t>SYSTEM exibe uma mensagem pop-up indicando que não existem extrações para serem deletadas</t>
   </si>
 </sst>
 </file>
@@ -263,7 +260,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="116.5390625" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="111.2421875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="79.53515625" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>
@@ -735,7 +732,7 @@
         <v>27</v>
       </c>
       <c r="D36" t="s" s="3">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s" s="3">
         <v>27</v>
@@ -755,7 +752,7 @@
         <v>27</v>
       </c>
       <c r="D37" t="s" s="3">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E37" t="s" s="3">
         <v>27</v>
@@ -777,7 +774,7 @@
         <v>11</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s" s="1">
         <v>13</v>
@@ -791,7 +788,7 @@
         <v>15</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E42" t="s" s="1">
         <v>17</v>
@@ -836,7 +833,7 @@
         <v>27</v>
       </c>
       <c r="D45" t="s" s="3">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E45" t="s" s="3">
         <v>27</v>
@@ -856,7 +853,7 @@
         <v>27</v>
       </c>
       <c r="D46" t="s" s="3">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E46" t="s" s="3">
         <v>27</v>

</xml_diff>